<commit_message>
[UI] 도감 UI, 슬롯 UI 구성
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Item.xlsx
+++ b/JsonConverter/ExcelFiles/Item.xlsx
@@ -14,123 +14,126 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
+  <x:si>
+    <x:t>Icon/Icon_Item_Box_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_Gold_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>착용하면 공격력이 강해진다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxStackCount</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Potato_1</x:t>
+  </x:si>
   <x:si>
     <x:t>딸기, 겨울에 더 맛있다.</x:t>
   </x:si>
   <x:si>
+    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SellingPrice</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_DummyBox_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>화폐</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>감자</x:t>
+  </x:si>
+  <x:si>
+    <x:t>옥수수</x:t>
+  </x:si>
+  <x:si>
+    <x:t>딸기</x:t>
+  </x:si>
+  <x:si>
+    <x:t>감자다. 딱히 의미가 있진 않다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_Item_Corn</x:t>
+  </x:si>
+  <x:si>
     <x:t>Item_Starwberry_1</x:t>
   </x:si>
   <x:si>
-    <x:t>딸기</x:t>
+    <x:t>상자다. 딱히 의미가 있진 않다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Item_Equip_Hat_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>옥수수다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Normal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grade</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Epic</x:t>
   </x:si>
   <x:si>
     <x:t>의문의 모자</x:t>
   </x:si>
   <x:si>
-    <x:t>Normal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Epic</x:t>
-  </x:si>
-  <x:si>
-    <x:t>옥수수다</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Grade</x:t>
-  </x:si>
-  <x:si>
     <x:t>Legend</x:t>
   </x:si>
   <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>화폐</x:t>
-  </x:si>
-  <x:si>
-    <x:t>상자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>옥수수</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>감자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>감자다. 딱히 의미가 있진 않다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Equip_Hat_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>상자다. 딱히 의미가 있진 않다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_Corn</x:t>
+    <x:t>캐릭터 고유 ID</x:t>
   </x:si>
   <x:si>
     <x:t>ItemType</x:t>
   </x:si>
   <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
+    <x:t>Item_Corn_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>지역에 나타나는 금화</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Equipment</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
   </x:si>
   <x:si>
     <x:t>Item_Gold_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Item_Corn_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>지역에 나타나는 금화</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Equipment</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_Potato_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SellingPrice</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Item_DummyBox_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>착용하면 공격력이 강해진다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MaxStackCount</x:t>
+    <x:t>Description</x:t>
   </x:si>
   <x:si>
     <x:t>Icon/Icon_Item_Equip_Hat_1</x:t>
   </x:si>
   <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_Gold_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_Item_Box_1</x:t>
+    <x:t>Icon/Icon_Item_Strawberry_1</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1426,87 +1429,88 @@
     <x:col min="2" max="2" width="19.5703125" style="2" customWidth="1"/>
     <x:col min="3" max="3" width="50.7109375" style="2" customWidth="1"/>
     <x:col min="4" max="4" width="26.5703125" style="2" customWidth="1"/>
-    <x:col min="5" max="7" width="12.5703125" style="2"/>
+    <x:col min="5" max="5" width="12.5703125" style="2"/>
+    <x:col min="6" max="7" width="12.5703125" style="2" bestFit="1" customWidth="1"/>
     <x:col min="8" max="8" width="28.42578125" style="2" customWidth="1"/>
     <x:col min="9" max="16384" width="12.5703125" style="2"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:8" ht="12.300000000000001">
       <x:c r="A2" s="1" t="s">
-        <x:v>11</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8" s="12" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="11" t="s">
-        <x:v>15</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="11" t="s">
-        <x:v>8</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C3" s="11" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="D3" s="14" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E3" s="13" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F3" s="13" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G3" s="13" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H3" s="13" t="s">
         <x:v>35</x:v>
-      </x:c>
-      <x:c r="D3" s="14" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E3" s="13" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="F3" s="13" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="G3" s="13" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="H3" s="13" t="s">
-        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>30</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D4" s="4" t="s">
-        <x:v>4</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E4" s="4" t="s">
-        <x:v>4</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F4" s="4">
         <x:v>20</x:v>
@@ -1515,7 +1519,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="H4" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I4" s="4"/>
       <x:c r="J4" s="4"/>
@@ -1525,19 +1529,19 @@
     </x:row>
     <x:row r="5" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>26</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
-        <x:v>4</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E5" s="4" t="s">
-        <x:v>10</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F5" s="4">
         <x:v>1000</x:v>
@@ -1546,7 +1550,7 @@
         <x:v>1000</x:v>
       </x:c>
       <x:c r="H5" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="4"/>
       <x:c r="J5" s="4"/>
@@ -1556,19 +1560,19 @@
     </x:row>
     <x:row r="6" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A6" s="5" t="s">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>3</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>31</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D6" s="4" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="E6" s="4" t="s">
         <x:v>27</x:v>
-      </x:c>
-      <x:c r="E6" s="4" t="s">
-        <x:v>6</x:v>
       </x:c>
       <x:c r="F6" s="4">
         <x:v>0</x:v>
@@ -1577,7 +1581,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H6" s="4" t="s">
-        <x:v>34</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="I6" s="4"/>
       <x:c r="K6" s="4"/>
@@ -1586,19 +1590,19 @@
     </x:row>
     <x:row r="7" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
-        <x:v>25</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>7</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D7" s="4" t="s">
-        <x:v>4</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E7" s="4" t="s">
-        <x:v>4</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F7" s="4">
         <x:v>100</x:v>
@@ -1607,7 +1611,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="H7" s="4" t="s">
-        <x:v>21</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="I7" s="4"/>
       <x:c r="J7" s="4"/>
@@ -1617,19 +1621,19 @@
     </x:row>
     <x:row r="8" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A8" s="15" t="s">
-        <x:v>28</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C8" s="3" t="s">
-        <x:v>18</x:v>
-      </x:c>
       <x:c r="D8" s="4" t="s">
-        <x:v>4</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E8" s="4" t="s">
-        <x:v>4</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F8" s="4">
         <x:v>20</x:v>
@@ -1638,7 +1642,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="H8" s="4" t="s">
-        <x:v>38</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I8" s="4"/>
       <x:c r="J8" s="4"/>
@@ -1648,19 +1652,29 @@
     </x:row>
     <x:row r="9" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A9" s="6" t="s">
-        <x:v>1</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B9" s="6" t="s">
-        <x:v>2</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C9" s="6" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D9" s="4"/>
-      <x:c r="E9" s="4"/>
-      <x:c r="F9" s="4"/>
-      <x:c r="G9" s="4"/>
-      <x:c r="H9" s="4"/>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F9" s="4">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G9" s="4">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="s">
+        <x:v>39</x:v>
+      </x:c>
       <x:c r="I9" s="4"/>
       <x:c r="J9" s="4"/>
       <x:c r="K9" s="4"/>

</xml_diff>